<commit_message>
Actualizar cortes programados de SEAL
</commit_message>
<xml_diff>
--- a/datos/cortes_programados.xlsx
+++ b/datos/cortes_programados.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cortes" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cortes" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cortes'!$A$1:$P$19</definedName>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-24 00:25:51</t>
+          <t>2026-10-24 09:51:57</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>C:\Users\MAJUEL~1\AppData\Local\Temp\msealk-extraccion-ej1anh1u</t>
+          <t>/tmp/msealk-extraccion-u3c582vl</t>
         </is>
       </c>
     </row>

</xml_diff>